<commit_message>
Modele des localites: X/Y facultatifs (notice)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B9L2AWyqvHA7ZfVpH7sJL9
</commit_message>
<xml_diff>
--- a/modele_localites_carte.xlsx
+++ b/modele_localites_carte.xlsx
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1570,11 +1573,10 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. Une ligne par localité : nom, X (longitude) et Y (latitude) en degrés décimaux WGS84 (ex. -4.856766 ; 5.503125).</t>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>1. Une ligne par localité : nom, puis X (longitude) et Y (latitude) en degrés décimaux WGS84 (ex. -4.856766 ; 5.503125). X et Y sont FACULTATIFS : laissés vides, la position est retrouvée automatiquement d'après le nom de la localité (zones habitées), en gardant l'homonyme le plus proche des parcelles de la coopérative. Une localité introuvable est signalée dans les contrôles : saisissez alors X et Y.</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1608,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>